<commit_message>
Actualizar analisis automatico 5min
</commit_message>
<xml_diff>
--- a/analisis_acciones.xlsx
+++ b/analisis_acciones.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z37"/>
+  <dimension ref="A1:AA37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,10 +539,15 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>Senal Bot</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>Razones</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Alertas</t>
         </is>
@@ -551,68 +556,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>COIN</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cripto / Trading</t>
+          <t>Equipos chips</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>216.6</v>
+        <v>421.22</v>
       </c>
       <c r="D2" t="n">
         <v>96</v>
       </c>
       <c r="E2" t="n">
-        <v>6.7</v>
+        <v>2.53</v>
       </c>
       <c r="F2" t="n">
-        <v>24.1</v>
+        <v>6.47</v>
       </c>
       <c r="G2" t="n">
-        <v>53.52</v>
+        <v>18.83</v>
       </c>
       <c r="H2" t="n">
-        <v>8.57</v>
+        <v>-4.98</v>
       </c>
       <c r="I2" t="n">
-        <v>1.31</v>
+        <v>0.61</v>
       </c>
       <c r="J2" t="n">
-        <v>12.22</v>
+        <v>18.91</v>
       </c>
       <c r="K2" t="n">
-        <v>5.64</v>
+        <v>4.49</v>
       </c>
       <c r="L2" t="n">
-        <v>212.32</v>
+        <v>414.6</v>
       </c>
       <c r="M2" t="n">
-        <v>218.43</v>
+        <v>424.06</v>
       </c>
       <c r="N2" t="n">
-        <v>200.11</v>
+        <v>395.69</v>
       </c>
       <c r="O2" t="n">
-        <v>243.48</v>
+        <v>462.82</v>
       </c>
       <c r="P2" t="n">
         <v>1.63</v>
       </c>
       <c r="Q2" t="n">
-        <v>61</v>
+        <v>54.9</v>
       </c>
       <c r="R2" t="n">
-        <v>9.42</v>
+        <v>4.19</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.57</v>
+        <v>-6.07</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -622,91 +627,96 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>🔥🔥🔥</t>
+          <t>🔥</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>COMPRA FUERTE</t>
+          <t>POSIBLE COMPRA</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; RSI saludable</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Tendencia larga débil; Momentum 5D extendido; Algo extendida sobre MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; RSI saludable</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Volumen bajo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IA / Chips</t>
+          <t>Equipos chips</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>428.43</v>
+        <v>283.1</v>
       </c>
       <c r="D3" t="n">
         <v>96</v>
       </c>
       <c r="E3" t="n">
-        <v>2.86</v>
+        <v>2.65</v>
       </c>
       <c r="F3" t="n">
-        <v>12.82</v>
+        <v>3.92</v>
       </c>
       <c r="G3" t="n">
-        <v>29.64</v>
+        <v>20.34</v>
       </c>
       <c r="H3" t="n">
-        <v>-2.71</v>
+        <v>-7.53</v>
       </c>
       <c r="I3" t="n">
-        <v>0.83</v>
+        <v>0.41</v>
       </c>
       <c r="J3" t="n">
-        <v>15.4</v>
+        <v>14.39</v>
       </c>
       <c r="K3" t="n">
-        <v>3.59</v>
+        <v>5.08</v>
       </c>
       <c r="L3" t="n">
-        <v>423.04</v>
+        <v>278.06</v>
       </c>
       <c r="M3" t="n">
-        <v>430.74</v>
+        <v>285.26</v>
       </c>
       <c r="N3" t="n">
-        <v>407.64</v>
+        <v>263.67</v>
       </c>
       <c r="O3" t="n">
-        <v>462.31</v>
+        <v>314.77</v>
       </c>
       <c r="P3" t="n">
         <v>1.63</v>
       </c>
       <c r="Q3" t="n">
-        <v>60.96</v>
+        <v>57.37</v>
       </c>
       <c r="R3" t="n">
-        <v>3.83</v>
+        <v>5.39</v>
       </c>
       <c r="S3" t="n">
-        <v>-2.11</v>
+        <v>-5.63</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -735,76 +745,81 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>MACD sin confirmar</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; RSI saludable</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Volumen bajo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9.48</v>
+        <v>1493.25</v>
       </c>
       <c r="D4" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E4" t="n">
-        <v>2.82</v>
+        <v>3.49</v>
       </c>
       <c r="F4" t="n">
-        <v>11.92</v>
+        <v>-1.44</v>
       </c>
       <c r="G4" t="n">
-        <v>-8.67</v>
+        <v>6.39</v>
       </c>
       <c r="H4" t="n">
-        <v>-3.61</v>
+        <v>-12.89</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9</v>
+        <v>0.66</v>
       </c>
       <c r="J4" t="n">
-        <v>0.43</v>
+        <v>60.71</v>
       </c>
       <c r="K4" t="n">
-        <v>4.57</v>
+        <v>4.07</v>
       </c>
       <c r="L4" t="n">
-        <v>9.33</v>
+        <v>1472</v>
       </c>
       <c r="M4" t="n">
-        <v>9.550000000000001</v>
+        <v>1502.36</v>
       </c>
       <c r="N4" t="n">
-        <v>8.890000000000001</v>
+        <v>1411.29</v>
       </c>
       <c r="O4" t="n">
-        <v>10.43</v>
+        <v>1626.81</v>
       </c>
       <c r="P4" t="n">
-        <v>1.61</v>
+        <v>1.63</v>
       </c>
       <c r="Q4" t="n">
-        <v>54.55</v>
+        <v>54.37</v>
       </c>
       <c r="R4" t="n">
-        <v>3.38</v>
+        <v>2.28</v>
       </c>
       <c r="S4" t="n">
-        <v>-4.63</v>
+        <v>-6.4</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -833,12 +848,17 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; RSI saludable</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>Tendencia larga débil; Débil vs QQQ</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; RSI saludable</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Volumen bajo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
@@ -854,55 +874,55 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>54.93</v>
+        <v>55.68</v>
       </c>
       <c r="D5" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E5" t="n">
-        <v>-1.26</v>
+        <v>-0.57</v>
       </c>
       <c r="F5" t="n">
-        <v>5.8</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>8.470000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="H5" t="n">
-        <v>-9.73</v>
+        <v>-3.31</v>
       </c>
       <c r="I5" t="n">
-        <v>0.68</v>
+        <v>0.38</v>
       </c>
       <c r="J5" t="n">
-        <v>1.69</v>
+        <v>1.62</v>
       </c>
       <c r="K5" t="n">
-        <v>3.08</v>
+        <v>2.91</v>
       </c>
       <c r="L5" t="n">
-        <v>54.34</v>
+        <v>55.11</v>
       </c>
       <c r="M5" t="n">
-        <v>55.18</v>
+        <v>55.92</v>
       </c>
       <c r="N5" t="n">
-        <v>52.65</v>
+        <v>53.49</v>
       </c>
       <c r="O5" t="n">
-        <v>58.65</v>
+        <v>59.25</v>
       </c>
       <c r="P5" t="n">
         <v>1.63</v>
       </c>
       <c r="Q5" t="n">
-        <v>58.59</v>
+        <v>55.66</v>
       </c>
       <c r="R5" t="n">
-        <v>1.08</v>
+        <v>2.06</v>
       </c>
       <c r="S5" t="n">
-        <v>-3.97</v>
+        <v>-2.66</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -927,10 +947,15 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
+        <is>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; RSI saludable</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
         <is>
           <t>MACD sin confirmar; Volumen bajo; Débil vs QQQ</t>
         </is>
@@ -939,7 +964,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -948,55 +973,55 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>212.65</v>
+        <v>392.55</v>
       </c>
       <c r="D6" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="E6" t="n">
-        <v>4.62</v>
+        <v>-0.47</v>
       </c>
       <c r="F6" t="n">
-        <v>34.95</v>
+        <v>3.33</v>
       </c>
       <c r="G6" t="n">
-        <v>74.03</v>
+        <v>7.45</v>
       </c>
       <c r="H6" t="n">
-        <v>19.42</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.89</v>
       </c>
       <c r="J6" t="n">
-        <v>18.49</v>
+        <v>15.57</v>
       </c>
       <c r="K6" t="n">
-        <v>8.699999999999999</v>
+        <v>3.97</v>
       </c>
       <c r="L6" t="n">
-        <v>206.18</v>
+        <v>387.1</v>
       </c>
       <c r="M6" t="n">
-        <v>215.42</v>
+        <v>394.89</v>
       </c>
       <c r="N6" t="n">
-        <v>187.69</v>
+        <v>371.53</v>
       </c>
       <c r="O6" t="n">
-        <v>253.33</v>
+        <v>426.81</v>
       </c>
       <c r="P6" t="n">
         <v>1.63</v>
       </c>
       <c r="Q6" t="n">
-        <v>60.64</v>
+        <v>52.36</v>
       </c>
       <c r="R6" t="n">
-        <v>7.33</v>
+        <v>0.15</v>
       </c>
       <c r="S6" t="n">
-        <v>-11.21</v>
+        <v>-6.54</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -1010,14 +1035,10 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>MEDIO</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>🔥🔥</t>
-        </is>
-      </c>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr">
         <is>
           <t>POSIBLE COMPRA</t>
@@ -1025,76 +1046,81 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>MACD sin confirmar; Algo extendida sobre MA20; Volatilidad alta</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; RSI saludable</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>MACD sin confirmar; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Equipos chips</t>
+          <t>Tecnología</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1845.19</v>
+        <v>264.04</v>
       </c>
       <c r="D7" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="E7" t="n">
-        <v>7.7</v>
+        <v>-3.48</v>
       </c>
       <c r="F7" t="n">
-        <v>4.32</v>
+        <v>6.03</v>
       </c>
       <c r="G7" t="n">
-        <v>27.35</v>
+        <v>32.82</v>
       </c>
       <c r="H7" t="n">
-        <v>-11.21</v>
+        <v>-5.42</v>
       </c>
       <c r="I7" t="n">
-        <v>1.16</v>
+        <v>0.43</v>
       </c>
       <c r="J7" t="n">
-        <v>83.20999999999999</v>
+        <v>7.26</v>
       </c>
       <c r="K7" t="n">
-        <v>4.51</v>
+        <v>2.75</v>
       </c>
       <c r="L7" t="n">
-        <v>1816.06</v>
+        <v>261.5</v>
       </c>
       <c r="M7" t="n">
-        <v>1857.67</v>
+        <v>265.13</v>
       </c>
       <c r="N7" t="n">
-        <v>1732.85</v>
+        <v>254.24</v>
       </c>
       <c r="O7" t="n">
-        <v>2028.26</v>
+        <v>280</v>
       </c>
       <c r="P7" t="n">
         <v>1.63</v>
       </c>
       <c r="Q7" t="n">
-        <v>54.45</v>
+        <v>60.15</v>
       </c>
       <c r="R7" t="n">
-        <v>2.61</v>
+        <v>0.86</v>
       </c>
       <c r="S7" t="n">
-        <v>-4.86</v>
+        <v>-5.21</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1108,14 +1134,10 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>MEDIO</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>🔥</t>
-        </is>
-      </c>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr">
         <is>
           <t>POSIBLE COMPRA</t>
@@ -1123,76 +1145,81 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>MACD sin confirmar; Momentum 5D extendido; Débil vs QQQ</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; RSI saludable</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>MACD sin confirmar; Volumen bajo; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SOUN</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>Energía</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8.449999999999999</v>
+        <v>150.85</v>
       </c>
       <c r="D8" t="n">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E8" t="n">
-        <v>-10.77</v>
+        <v>-2.6</v>
       </c>
       <c r="F8" t="n">
-        <v>23.54</v>
+        <v>1.08</v>
       </c>
       <c r="G8" t="n">
-        <v>13.27</v>
+        <v>1.62</v>
       </c>
       <c r="H8" t="n">
-        <v>8.01</v>
+        <v>-10.37</v>
       </c>
       <c r="I8" t="n">
-        <v>0.97</v>
+        <v>0.46</v>
       </c>
       <c r="J8" t="n">
-        <v>0.65</v>
+        <v>4.02</v>
       </c>
       <c r="K8" t="n">
-        <v>7.65</v>
+        <v>2.67</v>
       </c>
       <c r="L8" t="n">
-        <v>8.220000000000001</v>
+        <v>149.44</v>
       </c>
       <c r="M8" t="n">
-        <v>8.550000000000001</v>
+        <v>151.45</v>
       </c>
       <c r="N8" t="n">
-        <v>7.58</v>
+        <v>145.42</v>
       </c>
       <c r="O8" t="n">
-        <v>9.869999999999999</v>
+        <v>159.7</v>
       </c>
       <c r="P8" t="n">
         <v>1.63</v>
       </c>
       <c r="Q8" t="n">
-        <v>55.4</v>
+        <v>52.21</v>
       </c>
       <c r="R8" t="n">
-        <v>0.96</v>
+        <v>0.5</v>
       </c>
       <c r="S8" t="n">
-        <v>-15.88</v>
+        <v>-3.11</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -1206,14 +1233,10 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>MEDIO</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>🔥</t>
-        </is>
-      </c>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr">
         <is>
           <t>POSIBLE COMPRA</t>
@@ -1221,76 +1244,81 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; RSI saludable</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>Tendencia larga débil; Momentum negativo; Volatilidad alta</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; Tendencia larga positiva; RSI saludable; Histograma MACD mejora</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>MACD sin confirmar; Volumen bajo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>ETF Chips</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>404.54</v>
+        <v>503.79</v>
       </c>
       <c r="D9" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E9" t="n">
-        <v>0.73</v>
+        <v>4.36</v>
       </c>
       <c r="F9" t="n">
-        <v>9.460000000000001</v>
+        <v>25.56</v>
       </c>
       <c r="G9" t="n">
-        <v>10.21</v>
+        <v>42.14</v>
       </c>
       <c r="H9" t="n">
-        <v>-6.07</v>
+        <v>14.11</v>
       </c>
       <c r="I9" t="n">
-        <v>0.98</v>
+        <v>1.39</v>
       </c>
       <c r="J9" t="n">
-        <v>15.67</v>
+        <v>19.23</v>
       </c>
       <c r="K9" t="n">
-        <v>3.87</v>
+        <v>3.82</v>
       </c>
       <c r="L9" t="n">
-        <v>399.05</v>
+        <v>497.06</v>
       </c>
       <c r="M9" t="n">
-        <v>406.89</v>
+        <v>506.67</v>
       </c>
       <c r="N9" t="n">
-        <v>383.38</v>
+        <v>477.83</v>
       </c>
       <c r="O9" t="n">
-        <v>439.02</v>
+        <v>546.1</v>
       </c>
       <c r="P9" t="n">
         <v>1.63</v>
       </c>
       <c r="Q9" t="n">
-        <v>65.77</v>
+        <v>66.97</v>
       </c>
       <c r="R9" t="n">
-        <v>3.38</v>
+        <v>9.9</v>
       </c>
       <c r="S9" t="n">
-        <v>-3.68</v>
+        <v>-5.61</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -1307,7 +1335,11 @@
           <t>MEDIO</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>🔥🔥🔥</t>
+        </is>
+      </c>
       <c r="X9" t="inlineStr">
         <is>
           <t>POSIBLE COMPRA</t>
@@ -1315,77 +1347,82 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>RSI algo alto; Débil vs QQQ</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>RSI algo alto; Algo extendida sobre MA20</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Trading</t>
+          <t>ETF Mercado</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>80.78</v>
+        <v>734.6799999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="E10" t="n">
-        <v>5.53</v>
+        <v>1.51</v>
       </c>
       <c r="F10" t="n">
-        <v>12.71</v>
+        <v>5.79</v>
       </c>
       <c r="G10" t="n">
-        <v>13.58</v>
+        <v>8.06</v>
       </c>
       <c r="H10" t="n">
-        <v>-2.82</v>
+        <v>-5.66</v>
       </c>
       <c r="I10" t="n">
-        <v>0.74</v>
+        <v>0.58</v>
       </c>
       <c r="J10" t="n">
-        <v>4.22</v>
+        <v>6.74</v>
       </c>
       <c r="K10" t="n">
-        <v>5.23</v>
+        <v>0.92</v>
       </c>
       <c r="L10" t="n">
-        <v>79.3</v>
+        <v>732.3200000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>81.41</v>
+        <v>735.6900000000001</v>
       </c>
       <c r="N10" t="n">
-        <v>75.08</v>
+        <v>725.58</v>
       </c>
       <c r="O10" t="n">
-        <v>90.06999999999999</v>
+        <v>749.51</v>
       </c>
       <c r="P10" t="n">
         <v>1.63</v>
       </c>
       <c r="Q10" t="n">
-        <v>42.3</v>
+        <v>71.26000000000001</v>
       </c>
       <c r="R10" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="S10" t="n">
         <v>-0.82</v>
       </c>
-      <c r="S10" t="n">
-        <v>-13.44</v>
-      </c>
       <c r="T10" t="inlineStr">
         <is>
           <t>MEDIA</t>
@@ -1398,87 +1435,96 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>BAJO</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr"/>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>🔥</t>
+        </is>
+      </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>POSIBLE COMPRA</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; MA20 sobre MA50; MACD mejorando; Momentum 5D sano</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>Precio bajo MA20; Tendencia larga débil; MACD sin confirmar; Volumen bajo</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>RSI algo alto; Volumen bajo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>COIN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Espacial</t>
+          <t>Cripto / Trading</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>117.35</v>
+        <v>204.97</v>
       </c>
       <c r="D11" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="E11" t="n">
-        <v>46.12</v>
+        <v>3.65</v>
       </c>
       <c r="F11" t="n">
-        <v>66.17</v>
+        <v>11.15</v>
       </c>
       <c r="G11" t="n">
-        <v>77.78</v>
+        <v>24.74</v>
       </c>
       <c r="H11" t="n">
-        <v>50.64</v>
+        <v>-0.3</v>
       </c>
       <c r="I11" t="n">
-        <v>2.02</v>
+        <v>0.6</v>
       </c>
       <c r="J11" t="n">
-        <v>8.640000000000001</v>
+        <v>12.37</v>
       </c>
       <c r="K11" t="n">
-        <v>7.36</v>
+        <v>6.04</v>
       </c>
       <c r="L11" t="n">
-        <v>114.33</v>
+        <v>200.64</v>
       </c>
       <c r="M11" t="n">
-        <v>118.65</v>
+        <v>206.83</v>
       </c>
       <c r="N11" t="n">
-        <v>105.69</v>
+        <v>188.26</v>
       </c>
       <c r="O11" t="n">
-        <v>136.36</v>
+        <v>232.19</v>
       </c>
       <c r="P11" t="n">
         <v>1.63</v>
       </c>
       <c r="Q11" t="n">
-        <v>68.15000000000001</v>
+        <v>49.33</v>
       </c>
       <c r="R11" t="n">
-        <v>39.01</v>
+        <v>3.01</v>
       </c>
       <c r="S11" t="n">
-        <v>-5.32</v>
+        <v>-6.17</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -1492,7 +1538,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1502,81 +1548,86 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>POSIBLE COMPRA</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>RSI algo alto; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; RSI saludable; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Tendencia larga débil; Volumen bajo; Volatilidad alta</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>388.64</v>
+        <v>204.41</v>
       </c>
       <c r="D12" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="E12" t="n">
-        <v>1.41</v>
+        <v>-2.12</v>
       </c>
       <c r="F12" t="n">
-        <v>20.95</v>
+        <v>26.79</v>
       </c>
       <c r="G12" t="n">
-        <v>25.86</v>
+        <v>63.16</v>
       </c>
       <c r="H12" t="n">
-        <v>5.42</v>
+        <v>15.34</v>
       </c>
       <c r="I12" t="n">
-        <v>1.1</v>
+        <v>0.51</v>
       </c>
       <c r="J12" t="n">
-        <v>10.65</v>
+        <v>18.09</v>
       </c>
       <c r="K12" t="n">
-        <v>2.74</v>
+        <v>8.85</v>
       </c>
       <c r="L12" t="n">
-        <v>384.91</v>
+        <v>198.08</v>
       </c>
       <c r="M12" t="n">
-        <v>390.24</v>
+        <v>207.12</v>
       </c>
       <c r="N12" t="n">
-        <v>374.26</v>
+        <v>179.98</v>
       </c>
       <c r="O12" t="n">
-        <v>412.07</v>
+        <v>244.22</v>
       </c>
       <c r="P12" t="n">
         <v>1.63</v>
       </c>
       <c r="Q12" t="n">
-        <v>82.15000000000001</v>
+        <v>52.42</v>
       </c>
       <c r="R12" t="n">
-        <v>7.69</v>
+        <v>2.06</v>
       </c>
       <c r="S12" t="n">
-        <v>-3.32</v>
+        <v>-14.65</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
@@ -1590,7 +1641,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -1600,81 +1651,86 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>POSIBLE COMPRA</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado; Algo extendida sobre MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; RSI saludable</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>MACD sin confirmar; Volumen bajo; Volatilidad alta</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ETF Nasdaq</t>
+          <t>Autos / Tech</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>713.29</v>
+        <v>427.91</v>
       </c>
       <c r="D13" t="n">
         <v>86</v>
       </c>
       <c r="E13" t="n">
-        <v>6.01</v>
+        <v>9.9</v>
       </c>
       <c r="F13" t="n">
-        <v>15.53</v>
+        <v>17.49</v>
       </c>
       <c r="G13" t="n">
-        <v>18.9</v>
+        <v>2.51</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>6.04</v>
       </c>
       <c r="I13" t="n">
-        <v>0.88</v>
+        <v>0.65</v>
       </c>
       <c r="J13" t="n">
-        <v>9.84</v>
+        <v>16.76</v>
       </c>
       <c r="K13" t="n">
-        <v>1.38</v>
+        <v>3.92</v>
       </c>
       <c r="L13" t="n">
-        <v>709.84</v>
+        <v>422.04</v>
       </c>
       <c r="M13" t="n">
-        <v>714.77</v>
+        <v>430.42</v>
       </c>
       <c r="N13" t="n">
-        <v>700</v>
+        <v>405.28</v>
       </c>
       <c r="O13" t="n">
-        <v>734.95</v>
+        <v>464.78</v>
       </c>
       <c r="P13" t="n">
         <v>1.63</v>
       </c>
       <c r="Q13" t="n">
-        <v>86.72</v>
+        <v>66.81</v>
       </c>
       <c r="R13" t="n">
-        <v>7.17</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.18</v>
+        <v>-4.73</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -1688,7 +1744,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1698,81 +1754,86 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>POSIBLE COMPRA</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado; Momentum 5D extendido; Algo extendida sobre MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; MACD positivo; Fuerte vs QQQ</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Tendencia larga débil; RSI algo alto; Volumen bajo; Momentum 5D extendido; Algo extendida sobre MA20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Memoria / Chips</t>
+          <t>Tecnología</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>795.33</v>
+        <v>294.15</v>
       </c>
       <c r="D14" t="n">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E14" t="n">
-        <v>37.97</v>
+        <v>3.6</v>
       </c>
       <c r="F14" t="n">
-        <v>86.45</v>
+        <v>13.75</v>
       </c>
       <c r="G14" t="n">
-        <v>92.2</v>
+        <v>15.11</v>
       </c>
       <c r="H14" t="n">
-        <v>70.92</v>
+        <v>2.3</v>
       </c>
       <c r="I14" t="n">
-        <v>1.56</v>
+        <v>0.48</v>
       </c>
       <c r="J14" t="n">
-        <v>45.86</v>
+        <v>6.25</v>
       </c>
       <c r="K14" t="n">
-        <v>5.77</v>
+        <v>2.13</v>
       </c>
       <c r="L14" t="n">
-        <v>779.28</v>
+        <v>291.96</v>
       </c>
       <c r="M14" t="n">
-        <v>802.21</v>
+        <v>295.09</v>
       </c>
       <c r="N14" t="n">
-        <v>733.41</v>
+        <v>285.71</v>
       </c>
       <c r="O14" t="n">
-        <v>896.23</v>
+        <v>307.91</v>
       </c>
       <c r="P14" t="n">
         <v>1.63</v>
       </c>
       <c r="Q14" t="n">
-        <v>89.27</v>
+        <v>75.62</v>
       </c>
       <c r="R14" t="n">
-        <v>46.25</v>
+        <v>6.41</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.85</v>
+        <v>-0.25</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -1801,12 +1862,17 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado; Subida muy extendida 5D; Muy alejada de MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>RSI sobrecomprado; Volumen bajo</t>
         </is>
       </c>
     </row>
@@ -1822,55 +1888,55 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>219.44</v>
+        <v>218.52</v>
       </c>
       <c r="D15" t="n">
         <v>96</v>
       </c>
       <c r="E15" t="n">
-        <v>10.56</v>
+        <v>11.21</v>
       </c>
       <c r="F15" t="n">
-        <v>15.92</v>
+        <v>11.2</v>
       </c>
       <c r="G15" t="n">
-        <v>17.39</v>
+        <v>19.54</v>
       </c>
       <c r="H15" t="n">
-        <v>0.39</v>
+        <v>-0.25</v>
       </c>
       <c r="I15" t="n">
-        <v>1.03</v>
+        <v>0.71</v>
       </c>
       <c r="J15" t="n">
-        <v>7.7</v>
+        <v>8.08</v>
       </c>
       <c r="K15" t="n">
-        <v>3.51</v>
+        <v>3.7</v>
       </c>
       <c r="L15" t="n">
-        <v>216.75</v>
+        <v>215.69</v>
       </c>
       <c r="M15" t="n">
-        <v>220.59</v>
+        <v>219.73</v>
       </c>
       <c r="N15" t="n">
-        <v>209.05</v>
+        <v>207.62</v>
       </c>
       <c r="O15" t="n">
-        <v>236.37</v>
+        <v>236.29</v>
       </c>
       <c r="P15" t="n">
         <v>1.63</v>
       </c>
       <c r="Q15" t="n">
-        <v>64.92</v>
+        <v>62.54</v>
       </c>
       <c r="R15" t="n">
-        <v>7.21</v>
+        <v>6.19</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.29</v>
+        <v>-2.34</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -1895,80 +1961,85 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>Subida muy extendida 5D; Algo extendida sobre MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; RSI saludable</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Volumen bajo; Subida muy extendida 5D</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Equipos chips</t>
+          <t>ETF Nasdaq</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>443.62</v>
+        <v>700.5599999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E16" t="n">
-        <v>13.35</v>
+        <v>2.78</v>
       </c>
       <c r="F16" t="n">
-        <v>12.1</v>
+        <v>11.45</v>
       </c>
       <c r="G16" t="n">
-        <v>35.26</v>
+        <v>16.53</v>
       </c>
       <c r="H16" t="n">
-        <v>-3.43</v>
+        <v>-0</v>
       </c>
       <c r="I16" t="n">
-        <v>1.18</v>
+        <v>0.76</v>
       </c>
       <c r="J16" t="n">
-        <v>17.89</v>
+        <v>10.25</v>
       </c>
       <c r="K16" t="n">
-        <v>4.03</v>
+        <v>1.46</v>
       </c>
       <c r="L16" t="n">
-        <v>437.36</v>
+        <v>696.97</v>
       </c>
       <c r="M16" t="n">
-        <v>446.3</v>
+        <v>702.09</v>
       </c>
       <c r="N16" t="n">
-        <v>419.47</v>
+        <v>686.72</v>
       </c>
       <c r="O16" t="n">
-        <v>482.98</v>
+        <v>723.1</v>
       </c>
       <c r="P16" t="n">
         <v>1.63</v>
       </c>
       <c r="Q16" t="n">
-        <v>64.68000000000001</v>
+        <v>73.70999999999999</v>
       </c>
       <c r="R16" t="n">
-        <v>10.08</v>
+        <v>4.69</v>
       </c>
       <c r="S16" t="n">
-        <v>-1.08</v>
+        <v>-1.96</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1989,76 +2060,81 @@
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>Subida muy extendida 5D; Débil vs QQQ; Algo extendida sobre MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>RSI sobrecomprado</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Espacial</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1565.81</v>
+        <v>117.43</v>
       </c>
       <c r="D17" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="E17" t="n">
-        <v>12.96</v>
+        <v>49.09</v>
       </c>
       <c r="F17" t="n">
-        <v>4.6</v>
+        <v>62.59</v>
       </c>
       <c r="G17" t="n">
-        <v>11.54</v>
+        <v>74.12</v>
       </c>
       <c r="H17" t="n">
-        <v>-10.93</v>
+        <v>51.14</v>
       </c>
       <c r="I17" t="n">
-        <v>1.16</v>
+        <v>0.92</v>
       </c>
       <c r="J17" t="n">
-        <v>61.22</v>
+        <v>8.81</v>
       </c>
       <c r="K17" t="n">
-        <v>3.91</v>
+        <v>7.5</v>
       </c>
       <c r="L17" t="n">
-        <v>1544.38</v>
+        <v>114.34</v>
       </c>
       <c r="M17" t="n">
-        <v>1574.99</v>
+        <v>118.75</v>
       </c>
       <c r="N17" t="n">
-        <v>1483.16</v>
+        <v>105.54</v>
       </c>
       <c r="O17" t="n">
-        <v>1700.5</v>
+        <v>136.8</v>
       </c>
       <c r="P17" t="n">
         <v>1.63</v>
       </c>
       <c r="Q17" t="n">
-        <v>60.07</v>
+        <v>66.84999999999999</v>
       </c>
       <c r="R17" t="n">
-        <v>7.17</v>
+        <v>35.48</v>
       </c>
       <c r="S17" t="n">
-        <v>-1.85</v>
+        <v>-5.26</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
@@ -2083,19 +2159,24 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>Subida muy extendida 5D; Débil vs QQQ; Algo extendida sobre MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>RSI algo alto; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2104,55 +2185,55 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>292.68</v>
+        <v>384.89</v>
       </c>
       <c r="D18" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="E18" t="n">
-        <v>5.73</v>
+        <v>-0.91</v>
       </c>
       <c r="F18" t="n">
-        <v>12.92</v>
+        <v>15.61</v>
       </c>
       <c r="G18" t="n">
-        <v>11.83</v>
+        <v>25.98</v>
       </c>
       <c r="H18" t="n">
-        <v>-2.61</v>
+        <v>4.16</v>
       </c>
       <c r="I18" t="n">
-        <v>0.8</v>
+        <v>0.51</v>
       </c>
       <c r="J18" t="n">
-        <v>6.64</v>
+        <v>10.53</v>
       </c>
       <c r="K18" t="n">
-        <v>2.27</v>
+        <v>2.74</v>
       </c>
       <c r="L18" t="n">
-        <v>290.36</v>
+        <v>381.2</v>
       </c>
       <c r="M18" t="n">
-        <v>293.68</v>
+        <v>386.47</v>
       </c>
       <c r="N18" t="n">
-        <v>283.72</v>
+        <v>370.67</v>
       </c>
       <c r="O18" t="n">
-        <v>307.28</v>
+        <v>408.06</v>
       </c>
       <c r="P18" t="n">
         <v>1.63</v>
       </c>
       <c r="Q18" t="n">
-        <v>78.04000000000001</v>
+        <v>77.01000000000001</v>
       </c>
       <c r="R18" t="n">
-        <v>6.47</v>
+        <v>5.89</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.71</v>
+        <v>-4.26</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -2177,76 +2258,81 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>RSI sobrecomprado; Volumen bajo</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Equipos chips</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>296.05</v>
+        <v>116.66</v>
       </c>
       <c r="D19" t="n">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="E19" t="n">
-        <v>14.5</v>
+        <v>7.87</v>
       </c>
       <c r="F19" t="n">
-        <v>10.75</v>
+        <v>82.81999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>28.15</v>
+        <v>149.33</v>
       </c>
       <c r="H19" t="n">
-        <v>-4.78</v>
+        <v>71.37</v>
       </c>
       <c r="I19" t="n">
-        <v>0.86</v>
+        <v>0.83</v>
       </c>
       <c r="J19" t="n">
-        <v>13.7</v>
+        <v>9.15</v>
       </c>
       <c r="K19" t="n">
-        <v>4.63</v>
+        <v>7.84</v>
       </c>
       <c r="L19" t="n">
-        <v>291.25</v>
+        <v>113.46</v>
       </c>
       <c r="M19" t="n">
-        <v>298.11</v>
+        <v>118.03</v>
       </c>
       <c r="N19" t="n">
-        <v>277.55</v>
+        <v>104.31</v>
       </c>
       <c r="O19" t="n">
-        <v>326.19</v>
+        <v>136.79</v>
       </c>
       <c r="P19" t="n">
         <v>1.63</v>
       </c>
       <c r="Q19" t="n">
-        <v>66.63</v>
+        <v>77.66</v>
       </c>
       <c r="R19" t="n">
-        <v>10.43</v>
+        <v>29.3</v>
       </c>
       <c r="S19" t="n">
-        <v>-1.32</v>
+        <v>-12.12</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
@@ -2271,76 +2357,81 @@
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>RSI algo alto; Subida muy extendida 5D; Débil vs QQQ; Algo extendida sobre MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>RSI sobrecomprado; Momentum 5D extendido; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ETF Mercado</t>
+          <t>Servidores IA</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>739.3</v>
+        <v>32.13</v>
       </c>
       <c r="D20" t="n">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E20" t="n">
-        <v>2.97</v>
+        <v>15.45</v>
       </c>
       <c r="F20" t="n">
-        <v>7.75</v>
+        <v>18.13</v>
       </c>
       <c r="G20" t="n">
-        <v>8.81</v>
+        <v>5.21</v>
       </c>
       <c r="H20" t="n">
-        <v>-7.78</v>
+        <v>6.68</v>
       </c>
       <c r="I20" t="n">
-        <v>0.85</v>
+        <v>0.62</v>
       </c>
       <c r="J20" t="n">
-        <v>6.73</v>
+        <v>2.43</v>
       </c>
       <c r="K20" t="n">
-        <v>0.91</v>
+        <v>7.56</v>
       </c>
       <c r="L20" t="n">
-        <v>736.9400000000001</v>
+        <v>31.28</v>
       </c>
       <c r="M20" t="n">
-        <v>740.3099999999999</v>
+        <v>32.49</v>
       </c>
       <c r="N20" t="n">
-        <v>730.21</v>
+        <v>28.85</v>
       </c>
       <c r="O20" t="n">
-        <v>754.11</v>
+        <v>37.47</v>
       </c>
       <c r="P20" t="n">
         <v>1.63</v>
       </c>
       <c r="Q20" t="n">
-        <v>80.52</v>
+        <v>56.5</v>
       </c>
       <c r="R20" t="n">
-        <v>3.29</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.2</v>
+        <v>-11.66</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
@@ -2365,12 +2456,17 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado; Débil vs QQQ</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; RSI saludable; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Tendencia larga débil; Volumen bajo; Subida muy extendida 5D; Algo extendida sobre MA20; Volatilidad alta</t>
         </is>
       </c>
     </row>
@@ -2386,55 +2482,55 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>56.89</v>
+        <v>53.75</v>
       </c>
       <c r="D21" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="E21" t="n">
-        <v>24.35</v>
+        <v>11.98</v>
       </c>
       <c r="F21" t="n">
-        <v>91.16</v>
+        <v>50.31</v>
       </c>
       <c r="G21" t="n">
-        <v>81.76000000000001</v>
+        <v>57.58</v>
       </c>
       <c r="H21" t="n">
-        <v>75.63</v>
+        <v>38.86</v>
       </c>
       <c r="I21" t="n">
-        <v>1.47</v>
+        <v>0.78</v>
       </c>
       <c r="J21" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="K21" t="n">
-        <v>7.56</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="L21" t="n">
-        <v>55.38</v>
+        <v>52.14</v>
       </c>
       <c r="M21" t="n">
-        <v>57.54</v>
+        <v>54.44</v>
       </c>
       <c r="N21" t="n">
-        <v>51.08</v>
+        <v>47.54</v>
       </c>
       <c r="O21" t="n">
-        <v>66.34999999999999</v>
+        <v>63.86</v>
       </c>
       <c r="P21" t="n">
         <v>1.63</v>
       </c>
       <c r="Q21" t="n">
-        <v>65.56</v>
+        <v>58.84</v>
       </c>
       <c r="R21" t="n">
-        <v>23.87</v>
+        <v>14.79</v>
       </c>
       <c r="S21" t="n">
-        <v>-2.82</v>
+        <v>-9.130000000000001</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
@@ -2459,76 +2555,81 @@
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; MACD positivo</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>Tendencia larga débil; RSI algo alto; Subida muy extendida 5D; Muy alejada de MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; RSI saludable; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Tendencia larga débil; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ETF Chips</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>532.76</v>
+        <v>204.84</v>
       </c>
       <c r="D22" t="n">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E22" t="n">
-        <v>15.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>35.45</v>
+        <v>54.2</v>
       </c>
       <c r="G22" t="n">
-        <v>51.66</v>
+        <v>46.52</v>
       </c>
       <c r="H22" t="n">
-        <v>19.92</v>
+        <v>42.75</v>
       </c>
       <c r="I22" t="n">
-        <v>1.08</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>17.4</v>
+        <v>18.85</v>
       </c>
       <c r="K22" t="n">
-        <v>3.27</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L22" t="n">
-        <v>526.67</v>
+        <v>198.24</v>
       </c>
       <c r="M22" t="n">
-        <v>535.37</v>
+        <v>207.67</v>
       </c>
       <c r="N22" t="n">
-        <v>509.27</v>
+        <v>179.39</v>
       </c>
       <c r="O22" t="n">
-        <v>571.05</v>
+        <v>246.31</v>
       </c>
       <c r="P22" t="n">
         <v>1.63</v>
       </c>
       <c r="Q22" t="n">
-        <v>78.84999999999999</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="R22" t="n">
-        <v>17.53</v>
+        <v>23.4</v>
       </c>
       <c r="S22" t="n">
-        <v>-0.18</v>
+        <v>-17.37</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
@@ -2553,76 +2654,81 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado; Subida muy extendida 5D; Muy alejada de MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; MACD positivo; Fuerte vs QQQ</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Tendencia larga débil; RSI algo alto; Momentum 5D extendido; Muy alejada de MA20; Volatilidad muy alta</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>IA / Chips</t>
+          <t>Memoria / Chips</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>458.79</v>
+        <v>732.46</v>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="E23" t="n">
-        <v>34.33</v>
+        <v>14.41</v>
       </c>
       <c r="F23" t="n">
-        <v>85.87</v>
+        <v>57.3</v>
       </c>
       <c r="G23" t="n">
-        <v>122.78</v>
+        <v>78</v>
       </c>
       <c r="H23" t="n">
-        <v>70.34</v>
+        <v>45.85</v>
       </c>
       <c r="I23" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.13</v>
       </c>
       <c r="J23" t="n">
-        <v>27.39</v>
+        <v>49.16</v>
       </c>
       <c r="K23" t="n">
-        <v>5.97</v>
+        <v>6.71</v>
       </c>
       <c r="L23" t="n">
-        <v>449.2</v>
+        <v>715.26</v>
       </c>
       <c r="M23" t="n">
-        <v>462.9</v>
+        <v>739.83</v>
       </c>
       <c r="N23" t="n">
-        <v>421.82</v>
+        <v>666.1</v>
       </c>
       <c r="O23" t="n">
-        <v>519.04</v>
+        <v>840.61</v>
       </c>
       <c r="P23" t="n">
         <v>1.63</v>
       </c>
       <c r="Q23" t="n">
-        <v>80.33</v>
+        <v>76.31999999999999</v>
       </c>
       <c r="R23" t="n">
-        <v>36.21</v>
+        <v>31.46</v>
       </c>
       <c r="S23" t="n">
-        <v>-2.22</v>
+        <v>-10.53</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
@@ -2647,76 +2753,81 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado; Subida muy extendida 5D; Muy alejada de MA20</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>RSI sobrecomprado; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>IA / Chips</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>129.44</v>
+        <v>436.53</v>
       </c>
       <c r="D24" t="n">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E24" t="n">
-        <v>35.14</v>
+        <v>22.88</v>
       </c>
       <c r="F24" t="n">
-        <v>98.59</v>
+        <v>71.14</v>
       </c>
       <c r="G24" t="n">
-        <v>178.49</v>
+        <v>110.56</v>
       </c>
       <c r="H24" t="n">
-        <v>83.06</v>
+        <v>59.69</v>
       </c>
       <c r="I24" t="n">
-        <v>1.18</v>
+        <v>0.58</v>
       </c>
       <c r="J24" t="n">
-        <v>8.390000000000001</v>
+        <v>28.31</v>
       </c>
       <c r="K24" t="n">
-        <v>6.48</v>
+        <v>6.49</v>
       </c>
       <c r="L24" t="n">
-        <v>126.5</v>
+        <v>426.62</v>
       </c>
       <c r="M24" t="n">
-        <v>130.7</v>
+        <v>440.78</v>
       </c>
       <c r="N24" t="n">
-        <v>118.12</v>
+        <v>398.31</v>
       </c>
       <c r="O24" t="n">
-        <v>147.89</v>
+        <v>498.82</v>
       </c>
       <c r="P24" t="n">
         <v>1.63</v>
       </c>
       <c r="Q24" t="n">
-        <v>88.95</v>
+        <v>72.89</v>
       </c>
       <c r="R24" t="n">
-        <v>47.8</v>
+        <v>26.2</v>
       </c>
       <c r="S24" t="n">
-        <v>-2.49</v>
+        <v>-6.97</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
@@ -2741,76 +2852,81 @@
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
+          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>RSI sobrecomprado; Volumen bajo; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Servidores IA</t>
+          <t>Equipos chips</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>33.52</v>
+        <v>1766.88</v>
       </c>
       <c r="D25" t="n">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="E25" t="n">
-        <v>20.06</v>
+        <v>1.96</v>
       </c>
       <c r="F25" t="n">
-        <v>29.07</v>
+        <v>-1.62</v>
       </c>
       <c r="G25" t="n">
-        <v>10.15</v>
+        <v>20.83</v>
       </c>
       <c r="H25" t="n">
-        <v>13.54</v>
+        <v>-13.07</v>
       </c>
       <c r="I25" t="n">
-        <v>1.02</v>
+        <v>0.48</v>
       </c>
       <c r="J25" t="n">
-        <v>2.34</v>
+        <v>87.83</v>
       </c>
       <c r="K25" t="n">
-        <v>6.98</v>
+        <v>4.97</v>
       </c>
       <c r="L25" t="n">
-        <v>32.7</v>
+        <v>1736.14</v>
       </c>
       <c r="M25" t="n">
-        <v>33.87</v>
+        <v>1780.06</v>
       </c>
       <c r="N25" t="n">
-        <v>30.36</v>
+        <v>1648.3</v>
       </c>
       <c r="O25" t="n">
-        <v>38.66</v>
+        <v>1960.12</v>
       </c>
       <c r="P25" t="n">
         <v>1.63</v>
       </c>
       <c r="Q25" t="n">
-        <v>61.54</v>
+        <v>46.88</v>
       </c>
       <c r="R25" t="n">
-        <v>15.08</v>
+        <v>-1.67</v>
       </c>
       <c r="S25" t="n">
-        <v>-7.84</v>
+        <v>-8.890000000000001</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
@@ -2824,91 +2940,96 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>NO COMPRAR</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; RSI saludable</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>Tendencia larga débil; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
+          <t>Mercado ALCISTA; MA20 sobre MA50; Tendencia larga positiva; Momentum 5D sano</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; MACD sin confirmar; Volumen bajo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Autos / Tech</t>
+          <t>IA / Chips</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>445</v>
+        <v>412.11</v>
       </c>
       <c r="D26" t="n">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="E26" t="n">
-        <v>13.37</v>
+        <v>-3.57</v>
       </c>
       <c r="F26" t="n">
-        <v>26.27</v>
+        <v>8.23</v>
       </c>
       <c r="G26" t="n">
-        <v>6.7</v>
+        <v>27</v>
       </c>
       <c r="H26" t="n">
-        <v>10.74</v>
+        <v>-3.22</v>
       </c>
       <c r="I26" t="n">
-        <v>1.17</v>
+        <v>0.54</v>
       </c>
       <c r="J26" t="n">
-        <v>15.49</v>
+        <v>15.39</v>
       </c>
       <c r="K26" t="n">
-        <v>3.48</v>
+        <v>3.73</v>
       </c>
       <c r="L26" t="n">
-        <v>439.58</v>
+        <v>406.73</v>
       </c>
       <c r="M26" t="n">
-        <v>447.32</v>
+        <v>414.42</v>
       </c>
       <c r="N26" t="n">
-        <v>424.09</v>
+        <v>391.34</v>
       </c>
       <c r="O26" t="n">
-        <v>479.07</v>
+        <v>445.98</v>
       </c>
       <c r="P26" t="n">
         <v>1.63</v>
       </c>
       <c r="Q26" t="n">
-        <v>78.11</v>
+        <v>45.45</v>
       </c>
       <c r="R26" t="n">
-        <v>13.7</v>
+        <v>-0.5</v>
       </c>
       <c r="S26" t="n">
-        <v>-0.93</v>
+        <v>-5.84</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -2918,91 +3039,96 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>NO COMPRAR</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; MACD positivo</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>Tendencia larga débil; RSI sobrecomprado; Subida muy extendida 5D; Muy alejada de MA20</t>
+          <t>Mercado ALCISTA; MA20 sobre MA50; Tendencia larga positiva</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; MACD sin confirmar; Volumen bajo; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>IA</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>268.99</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="D27" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="E27" t="n">
-        <v>-1.12</v>
+        <v>-5.58</v>
       </c>
       <c r="F27" t="n">
-        <v>12.13</v>
+        <v>5.77</v>
       </c>
       <c r="G27" t="n">
-        <v>34.76</v>
+        <v>-17.58</v>
       </c>
       <c r="H27" t="n">
-        <v>-3.4</v>
+        <v>-5.68</v>
       </c>
       <c r="I27" t="n">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="J27" t="n">
-        <v>7.23</v>
+        <v>0.46</v>
       </c>
       <c r="K27" t="n">
-        <v>2.69</v>
+        <v>5.21</v>
       </c>
       <c r="L27" t="n">
-        <v>266.46</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="M27" t="n">
-        <v>270.07</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N27" t="n">
-        <v>259.23</v>
+        <v>8.26</v>
       </c>
       <c r="O27" t="n">
-        <v>284.9</v>
+        <v>9.9</v>
       </c>
       <c r="P27" t="n">
-        <v>1.63</v>
+        <v>1.62</v>
       </c>
       <c r="Q27" t="n">
-        <v>72.06</v>
+        <v>42.75</v>
       </c>
       <c r="R27" t="n">
-        <v>3.04</v>
+        <v>-3.36</v>
       </c>
       <c r="S27" t="n">
-        <v>-3.44</v>
+        <v>-10.61</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>BAJA</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3012,87 +3138,92 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>NO COMPRAR</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; Tendencia larga positiva</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>RSI sobrecomprado; MACD sin confirmar; Débil vs QQQ</t>
+          <t>Mercado ALCISTA; MA20 sobre MA50; MACD positivo</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; Momentum negativo; Débil vs QQQ; Lejos del máximo 20D</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Energía</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>237.53</v>
+        <v>186.6</v>
       </c>
       <c r="D28" t="n">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="E28" t="n">
-        <v>41.07</v>
+        <v>-3.14</v>
       </c>
       <c r="F28" t="n">
-        <v>80.98999999999999</v>
+        <v>-0.22</v>
       </c>
       <c r="G28" t="n">
-        <v>72.64</v>
+        <v>2.55</v>
       </c>
       <c r="H28" t="n">
-        <v>65.45999999999999</v>
+        <v>-11.67</v>
       </c>
       <c r="I28" t="n">
-        <v>1.73</v>
+        <v>0.36</v>
       </c>
       <c r="J28" t="n">
-        <v>16.45</v>
+        <v>4.52</v>
       </c>
       <c r="K28" t="n">
-        <v>6.93</v>
+        <v>2.42</v>
       </c>
       <c r="L28" t="n">
-        <v>231.77</v>
+        <v>185.02</v>
       </c>
       <c r="M28" t="n">
-        <v>240</v>
+        <v>187.28</v>
       </c>
       <c r="N28" t="n">
-        <v>215.32</v>
+        <v>180.49</v>
       </c>
       <c r="O28" t="n">
-        <v>273.72</v>
+        <v>196.55</v>
       </c>
       <c r="P28" t="n">
         <v>1.63</v>
       </c>
       <c r="Q28" t="n">
-        <v>89.48</v>
+        <v>50.42</v>
       </c>
       <c r="R28" t="n">
-        <v>46.26</v>
+        <v>-0.22</v>
       </c>
       <c r="S28" t="n">
-        <v>-4.18</v>
+        <v>-3.88</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
@@ -3106,30 +3237,35 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>NO COMPRAR</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Precio sobre MA20; MA20 sobre MA50; MACD positivo</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>Tendencia larga débil; RSI sobrecomprado; Subida muy extendida 5D; Muy alejada de MA20</t>
+          <t>Mercado ALCISTA; Tendencia larga positiva; RSI saludable; Histograma MACD mejora</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; MACD sin confirmar; Volumen bajo; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>OXY</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3138,55 +3274,55 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>149.68</v>
+        <v>56.18</v>
       </c>
       <c r="D29" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="E29" t="n">
-        <v>-2.61</v>
+        <v>-5.33</v>
       </c>
       <c r="F29" t="n">
-        <v>-1.94</v>
+        <v>1.44</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.17</v>
+        <v>22.52</v>
       </c>
       <c r="H29" t="n">
-        <v>-17.47</v>
+        <v>-10.01</v>
       </c>
       <c r="I29" t="n">
-        <v>0.82</v>
+        <v>0.44</v>
       </c>
       <c r="J29" t="n">
-        <v>4.05</v>
+        <v>1.87</v>
       </c>
       <c r="K29" t="n">
-        <v>2.71</v>
+        <v>3.32</v>
       </c>
       <c r="L29" t="n">
-        <v>148.26</v>
+        <v>55.53</v>
       </c>
       <c r="M29" t="n">
-        <v>150.29</v>
+        <v>56.46</v>
       </c>
       <c r="N29" t="n">
-        <v>144.21</v>
+        <v>53.66</v>
       </c>
       <c r="O29" t="n">
-        <v>158.59</v>
+        <v>60.29</v>
       </c>
       <c r="P29" t="n">
         <v>1.63</v>
       </c>
       <c r="Q29" t="n">
-        <v>52.17</v>
+        <v>47.73</v>
       </c>
       <c r="R29" t="n">
-        <v>-0.22</v>
+        <v>-1.29</v>
       </c>
       <c r="S29" t="n">
-        <v>-3.86</v>
+        <v>-7.58</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
@@ -3211,80 +3347,85 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Tendencia larga positiva; RSI saludable; MACD mejorando</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>Precio bajo MA20; MACD sin confirmar; Débil vs QQQ</t>
+          <t>Mercado ALCISTA; Tendencia larga positiva; Histograma MACD mejora</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; MACD sin confirmar; Volumen bajo; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Energía</t>
+          <t>Pagos</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>184.74</v>
+        <v>45.68</v>
       </c>
       <c r="D30" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="E30" t="n">
-        <v>-3.92</v>
+        <v>-1.74</v>
       </c>
       <c r="F30" t="n">
-        <v>-3.67</v>
+        <v>-4.77</v>
       </c>
       <c r="G30" t="n">
-        <v>2.27</v>
+        <v>13.72</v>
       </c>
       <c r="H30" t="n">
-        <v>-19.2</v>
+        <v>-16.22</v>
       </c>
       <c r="I30" t="n">
-        <v>1.16</v>
+        <v>1.06</v>
       </c>
       <c r="J30" t="n">
-        <v>4.61</v>
+        <v>1.61</v>
       </c>
       <c r="K30" t="n">
-        <v>2.49</v>
+        <v>3.52</v>
       </c>
       <c r="L30" t="n">
-        <v>183.13</v>
+        <v>45.12</v>
       </c>
       <c r="M30" t="n">
-        <v>185.43</v>
+        <v>45.92</v>
       </c>
       <c r="N30" t="n">
-        <v>178.52</v>
+        <v>43.51</v>
       </c>
       <c r="O30" t="n">
-        <v>194.88</v>
+        <v>49.22</v>
       </c>
       <c r="P30" t="n">
         <v>1.63</v>
       </c>
       <c r="Q30" t="n">
-        <v>48.05</v>
+        <v>25.74</v>
       </c>
       <c r="R30" t="n">
-        <v>-1.23</v>
+        <v>-6.81</v>
       </c>
       <c r="S30" t="n">
-        <v>-4.84</v>
+        <v>-12.66</v>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>BAJA</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3305,12 +3446,17 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Tendencia larga positiva; RSI saludable; MACD mejorando</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Mercado ALCISTA; MA20 sobre MA50; Histograma MACD mejora</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
         </is>
       </c>
     </row>
@@ -3326,59 +3472,59 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>412.66</v>
+        <v>409.3</v>
       </c>
       <c r="D31" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.23</v>
+        <v>-0.51</v>
       </c>
       <c r="F31" t="n">
-        <v>7.36</v>
+        <v>4.12</v>
       </c>
       <c r="G31" t="n">
-        <v>2.93</v>
+        <v>2.22</v>
       </c>
       <c r="H31" t="n">
-        <v>-8.17</v>
+        <v>-7.33</v>
       </c>
       <c r="I31" t="n">
-        <v>0.96</v>
+        <v>0.45</v>
       </c>
       <c r="J31" t="n">
-        <v>11.8</v>
+        <v>11.72</v>
       </c>
       <c r="K31" t="n">
         <v>2.86</v>
       </c>
       <c r="L31" t="n">
-        <v>408.53</v>
+        <v>405.2</v>
       </c>
       <c r="M31" t="n">
-        <v>414.43</v>
+        <v>411.06</v>
       </c>
       <c r="N31" t="n">
-        <v>396.73</v>
+        <v>393.48</v>
       </c>
       <c r="O31" t="n">
-        <v>438.62</v>
+        <v>435.08</v>
       </c>
       <c r="P31" t="n">
         <v>1.63</v>
       </c>
       <c r="Q31" t="n">
-        <v>43.47</v>
+        <v>35.72</v>
       </c>
       <c r="R31" t="n">
-        <v>-1.17</v>
+        <v>-2.17</v>
       </c>
       <c r="S31" t="n">
-        <v>-4.85</v>
+        <v>-5.63</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>BAJA</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3399,76 +3545,81 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
+          <t>SELL / EVITAR</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
           <t>Mercado ALCISTA; MA20 sobre MA50</t>
         </is>
       </c>
-      <c r="Z31" t="inlineStr">
-        <is>
-          <t>Precio bajo MA20; Tendencia larga débil; MACD sin confirmar; Débil vs QQQ</t>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar; Volumen bajo</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>OXY</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Energía</t>
+          <t>Trading</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>55.14</v>
+        <v>77.72</v>
       </c>
       <c r="D32" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E32" t="n">
-        <v>-8.51</v>
+        <v>0.9</v>
       </c>
       <c r="F32" t="n">
-        <v>-5.03</v>
+        <v>-1.73</v>
       </c>
       <c r="G32" t="n">
-        <v>21.79</v>
+        <v>2.3</v>
       </c>
       <c r="H32" t="n">
-        <v>-20.56</v>
+        <v>-13.18</v>
       </c>
       <c r="I32" t="n">
-        <v>1.04</v>
+        <v>0.34</v>
       </c>
       <c r="J32" t="n">
-        <v>1.85</v>
+        <v>4.26</v>
       </c>
       <c r="K32" t="n">
-        <v>3.36</v>
+        <v>5.49</v>
       </c>
       <c r="L32" t="n">
-        <v>54.49</v>
+        <v>76.23</v>
       </c>
       <c r="M32" t="n">
-        <v>55.42</v>
+        <v>78.36</v>
       </c>
       <c r="N32" t="n">
-        <v>52.64</v>
+        <v>71.95999999999999</v>
       </c>
       <c r="O32" t="n">
-        <v>59.21</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="P32" t="n">
         <v>1.63</v>
       </c>
       <c r="Q32" t="n">
-        <v>46.84</v>
+        <v>35.81</v>
       </c>
       <c r="R32" t="n">
-        <v>-3.05</v>
+        <v>-4.49</v>
       </c>
       <c r="S32" t="n">
-        <v>-9.289999999999999</v>
+        <v>-16.72</v>
       </c>
       <c r="T32" t="inlineStr">
         <is>
@@ -3493,76 +3644,81 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; Tendencia larga positiva; MACD mejorando</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Mercado ALCISTA; MA20 sobre MA50; Histograma MACD mejora</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar; Volumen bajo</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>Tecnología</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>16.26</v>
+        <v>599.88</v>
       </c>
       <c r="D33" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E33" t="n">
-        <v>0.37</v>
+        <v>-0.84</v>
       </c>
       <c r="F33" t="n">
-        <v>-4.63</v>
+        <v>-9.449999999999999</v>
       </c>
       <c r="G33" t="n">
-        <v>-15.75</v>
+        <v>-6.15</v>
       </c>
       <c r="H33" t="n">
-        <v>-20.16</v>
+        <v>-20.9</v>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>0.44</v>
       </c>
       <c r="J33" t="n">
-        <v>0.82</v>
+        <v>18.43</v>
       </c>
       <c r="K33" t="n">
-        <v>5.02</v>
+        <v>3.07</v>
       </c>
       <c r="L33" t="n">
-        <v>15.97</v>
+        <v>593.4299999999999</v>
       </c>
       <c r="M33" t="n">
-        <v>16.38</v>
+        <v>602.64</v>
       </c>
       <c r="N33" t="n">
-        <v>15.16</v>
+        <v>575</v>
       </c>
       <c r="O33" t="n">
-        <v>18.06</v>
+        <v>640.4299999999999</v>
       </c>
       <c r="P33" t="n">
-        <v>1.64</v>
+        <v>1.63</v>
       </c>
       <c r="Q33" t="n">
-        <v>32.4</v>
+        <v>23.8</v>
       </c>
       <c r="R33" t="n">
-        <v>-7.35</v>
+        <v>-6.84</v>
       </c>
       <c r="S33" t="n">
-        <v>-19.23</v>
+        <v>-13.25</v>
       </c>
       <c r="T33" t="inlineStr">
         <is>
@@ -3587,76 +3743,81 @@
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; MA20 sobre MA50; MACD mejorando</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Mercado ALCISTA; MA20 sobre MA50; Histograma MACD mejora</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar; Volumen bajo</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IA / Software</t>
+          <t>Fintech</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>136.89</v>
+        <v>15.72</v>
       </c>
       <c r="D34" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E34" t="n">
-        <v>-6.26</v>
+        <v>-1.9</v>
       </c>
       <c r="F34" t="n">
-        <v>3.41</v>
+        <v>-12.26</v>
       </c>
       <c r="G34" t="n">
-        <v>6.01</v>
+        <v>-19.86</v>
       </c>
       <c r="H34" t="n">
-        <v>-12.12</v>
+        <v>-23.71</v>
       </c>
       <c r="I34" t="n">
-        <v>0.89</v>
+        <v>0.62</v>
       </c>
       <c r="J34" t="n">
-        <v>6.24</v>
+        <v>0.83</v>
       </c>
       <c r="K34" t="n">
-        <v>4.56</v>
+        <v>5.27</v>
       </c>
       <c r="L34" t="n">
-        <v>134.71</v>
+        <v>15.43</v>
       </c>
       <c r="M34" t="n">
-        <v>137.83</v>
+        <v>15.84</v>
       </c>
       <c r="N34" t="n">
-        <v>128.47</v>
+        <v>14.6</v>
       </c>
       <c r="O34" t="n">
-        <v>150.62</v>
+        <v>17.54</v>
       </c>
       <c r="P34" t="n">
-        <v>1.63</v>
+        <v>1.64</v>
       </c>
       <c r="Q34" t="n">
-        <v>40.84</v>
+        <v>28.04</v>
       </c>
       <c r="R34" t="n">
-        <v>-3.23</v>
+        <v>-9.9</v>
       </c>
       <c r="S34" t="n">
-        <v>-10.34</v>
+        <v>-21.93</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
@@ -3681,76 +3842,81 @@
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; MACD mejorando</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>Precio bajo MA20; Tendencia larga débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Mercado ALCISTA; MA20 sobre MA50; Histograma MACD mejora</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar; Volumen bajo</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>IA / Software</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>598.86</v>
+        <v>134.46</v>
       </c>
       <c r="D35" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E35" t="n">
-        <v>-1.89</v>
+        <v>-1.07</v>
       </c>
       <c r="F35" t="n">
-        <v>-5.62</v>
+        <v>-0.92</v>
       </c>
       <c r="G35" t="n">
-        <v>-7.76</v>
+        <v>2.32</v>
       </c>
       <c r="H35" t="n">
-        <v>-21.15</v>
+        <v>-12.37</v>
       </c>
       <c r="I35" t="n">
-        <v>0.92</v>
+        <v>0.49</v>
       </c>
       <c r="J35" t="n">
-        <v>18.32</v>
+        <v>6.04</v>
       </c>
       <c r="K35" t="n">
-        <v>3.06</v>
+        <v>4.5</v>
       </c>
       <c r="L35" t="n">
-        <v>592.45</v>
+        <v>132.34</v>
       </c>
       <c r="M35" t="n">
-        <v>601.61</v>
+        <v>135.36</v>
       </c>
       <c r="N35" t="n">
-        <v>574.13</v>
+        <v>126.3</v>
       </c>
       <c r="O35" t="n">
-        <v>639.17</v>
+        <v>147.75</v>
       </c>
       <c r="P35" t="n">
         <v>1.63</v>
       </c>
       <c r="Q35" t="n">
-        <v>26.31</v>
+        <v>29.98</v>
       </c>
       <c r="R35" t="n">
-        <v>-7.45</v>
+        <v>-4.9</v>
       </c>
       <c r="S35" t="n">
-        <v>-13.4</v>
+        <v>-11.94</v>
       </c>
       <c r="T35" t="inlineStr">
         <is>
@@ -3775,76 +3941,81 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; MA20 sobre MA50</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Mercado ALCISTA</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar; Volumen bajo</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>SOUN</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Pagos</t>
+          <t>IA</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>45.07</v>
+        <v>8.01</v>
       </c>
       <c r="D36" t="n">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="E36" t="n">
-        <v>-10.56</v>
+        <v>-12.36</v>
       </c>
       <c r="F36" t="n">
-        <v>-5.14</v>
+        <v>14.92</v>
       </c>
       <c r="G36" t="n">
-        <v>15.68</v>
+        <v>7.37</v>
       </c>
       <c r="H36" t="n">
-        <v>-20.67</v>
+        <v>3.47</v>
       </c>
       <c r="I36" t="n">
-        <v>1.12</v>
+        <v>0.6</v>
       </c>
       <c r="J36" t="n">
-        <v>1.56</v>
+        <v>0.65</v>
       </c>
       <c r="K36" t="n">
-        <v>3.46</v>
+        <v>8.08</v>
       </c>
       <c r="L36" t="n">
-        <v>44.52</v>
+        <v>7.78</v>
       </c>
       <c r="M36" t="n">
-        <v>45.3</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="N36" t="n">
-        <v>42.96</v>
+        <v>7.14</v>
       </c>
       <c r="O36" t="n">
-        <v>48.5</v>
+        <v>9.43</v>
       </c>
       <c r="P36" t="n">
         <v>1.63</v>
       </c>
       <c r="Q36" t="n">
-        <v>23.95</v>
+        <v>48.13</v>
       </c>
       <c r="R36" t="n">
-        <v>-8.27</v>
+        <v>-4.89</v>
       </c>
       <c r="S36" t="n">
-        <v>-13.82</v>
+        <v>-20.26</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
@@ -3858,7 +4029,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="W36" t="inlineStr"/>
@@ -3869,12 +4040,17 @@
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>Mercado ALCISTA; MA20 sobre MA50</t>
+          <t>SELL / EVITAR</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Mercado ALCISTA; MA20 sobre MA50; RSI saludable; Fuerte vs QQQ</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; MACD sin confirmar; Volumen bajo; Momentum negativo</t>
         </is>
       </c>
     </row>
@@ -3890,55 +4066,55 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>28.69</v>
+        <v>27.92</v>
       </c>
       <c r="D37" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E37" t="n">
-        <v>-10.57</v>
+        <v>-10.43</v>
       </c>
       <c r="F37" t="n">
-        <v>2.25</v>
+        <v>-5.45</v>
       </c>
       <c r="G37" t="n">
-        <v>-4.97</v>
+        <v>-9</v>
       </c>
       <c r="H37" t="n">
-        <v>-13.28</v>
+        <v>-16.9</v>
       </c>
       <c r="I37" t="n">
-        <v>0.74</v>
+        <v>0.4</v>
       </c>
       <c r="J37" t="n">
-        <v>1.81</v>
+        <v>1.76</v>
       </c>
       <c r="K37" t="n">
-        <v>6.31</v>
+        <v>6.32</v>
       </c>
       <c r="L37" t="n">
-        <v>28.06</v>
+        <v>27.3</v>
       </c>
       <c r="M37" t="n">
-        <v>28.96</v>
+        <v>28.18</v>
       </c>
       <c r="N37" t="n">
-        <v>26.25</v>
+        <v>25.54</v>
       </c>
       <c r="O37" t="n">
-        <v>32.67</v>
+        <v>31.8</v>
       </c>
       <c r="P37" t="n">
         <v>1.63</v>
       </c>
       <c r="Q37" t="n">
-        <v>33.95</v>
+        <v>24.32</v>
       </c>
       <c r="R37" t="n">
-        <v>-10.21</v>
+        <v>-12.4</v>
       </c>
       <c r="S37" t="n">
-        <v>-19.86</v>
+        <v>-22.01</v>
       </c>
       <c r="T37" t="inlineStr">
         <is>
@@ -3963,12 +4139,17 @@
       </c>
       <c r="Y37" t="inlineStr">
         <is>
+          <t>SELL / EVITAR</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
           <t>Mercado ALCISTA; MA20 sobre MA50</t>
         </is>
       </c>
-      <c r="Z37" t="inlineStr">
-        <is>
-          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar; Volumen bajo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar analisis automatico BOT-ARQ v4 paper
</commit_message>
<xml_diff>
--- a/analisis_acciones.xlsx
+++ b/analisis_acciones.xlsx
@@ -14683,7 +14683,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>BTC-USD -14.97% · ETH-USD -15.83%</t>
+          <t>BTC-USD -14.87% · ETH-USD -15.74%</t>
         </is>
       </c>
       <c r="X124" t="inlineStr">
@@ -14713,7 +14713,7 @@
       </c>
       <c r="AC124" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.83%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.87% · ETH-USD -15.74%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD124" t="n">
@@ -14799,7 +14799,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>BTC-USD -14.97% · ETH-USD -15.83%</t>
+          <t>BTC-USD -14.87% · ETH-USD -15.74%</t>
         </is>
       </c>
       <c r="X125" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="AC125" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.83%; MACD sin confirmar; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.87% · ETH-USD -15.74%; MACD sin confirmar; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD125" t="n">
@@ -28811,7 +28811,7 @@
       </c>
       <c r="W248" t="inlineStr">
         <is>
-          <t>BTC-USD -14.97% · ETH-USD -15.83%</t>
+          <t>BTC-USD -14.87% · ETH-USD -15.74%</t>
         </is>
       </c>
       <c r="X248" t="inlineStr">
@@ -28837,7 +28837,7 @@
       </c>
       <c r="AC248" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.83%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
+          <t>Sector no acompaña: BTC-USD -14.87% · ETH-USD -15.74%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD248" t="n">
@@ -31955,7 +31955,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>BTC-USD -14.97% · ETH-USD -15.83%</t>
+          <t>BTC-USD -14.87% · ETH-USD -15.74%</t>
         </is>
       </c>
       <c r="X276" t="inlineStr">
@@ -31981,7 +31981,7 @@
       </c>
       <c r="AC276" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.83%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: BTC-USD -14.87% · ETH-USD -15.74%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD276" t="n">

</xml_diff>

<commit_message>
Subir BOT-ARQ V4.1 Dashboard Cleanup Pro
</commit_message>
<xml_diff>
--- a/analisis_acciones.xlsx
+++ b/analisis_acciones.xlsx
@@ -14683,7 +14683,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>BTC-USD -14.87% · ETH-USD -15.74%</t>
+          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
         </is>
       </c>
       <c r="X124" t="inlineStr">
@@ -14713,7 +14713,7 @@
       </c>
       <c r="AC124" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.87% · ETH-USD -15.74%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD124" t="n">
@@ -14799,7 +14799,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>BTC-USD -14.87% · ETH-USD -15.74%</t>
+          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
         </is>
       </c>
       <c r="X125" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="AC125" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.87% · ETH-USD -15.74%; MACD sin confirmar; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; MACD sin confirmar; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD125" t="n">
@@ -14915,7 +14915,7 @@
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X126" t="inlineStr">
@@ -14945,7 +14945,7 @@
       </c>
       <c r="AC126" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD126" t="n">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X127" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="AC127" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD127" t="n">
@@ -18255,7 +18255,7 @@
       </c>
       <c r="W155" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X155" t="inlineStr">
@@ -18285,7 +18285,7 @@
       </c>
       <c r="AC155" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD155" t="n">
@@ -28023,7 +28023,7 @@
       </c>
       <c r="W241" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X241" t="inlineStr">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="AC241" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD241" t="n">
@@ -28139,7 +28139,7 @@
       </c>
       <c r="W242" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X242" t="inlineStr">
@@ -28165,7 +28165,7 @@
       </c>
       <c r="AC242" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Débil vs QQQ; Lejos del máximo 20D</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Débil vs QQQ; Lejos del máximo 20D</t>
         </is>
       </c>
       <c r="AD242" t="n">
@@ -28251,7 +28251,7 @@
       </c>
       <c r="W243" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X243" t="inlineStr">
@@ -28277,7 +28277,7 @@
       </c>
       <c r="AC243" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD243" t="n">
@@ -28363,7 +28363,7 @@
       </c>
       <c r="W244" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X244" t="inlineStr">
@@ -28389,7 +28389,7 @@
       </c>
       <c r="AC244" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD244" t="n">
@@ -28475,7 +28475,7 @@
       </c>
       <c r="W245" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X245" t="inlineStr">
@@ -28501,7 +28501,7 @@
       </c>
       <c r="AC245" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD245" t="n">
@@ -28587,7 +28587,7 @@
       </c>
       <c r="W246" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X246" t="inlineStr">
@@ -28613,7 +28613,7 @@
       </c>
       <c r="AC246" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD246" t="n">
@@ -28699,7 +28699,7 @@
       </c>
       <c r="W247" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X247" t="inlineStr">
@@ -28725,7 +28725,7 @@
       </c>
       <c r="AC247" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD247" t="n">
@@ -28811,7 +28811,7 @@
       </c>
       <c r="W248" t="inlineStr">
         <is>
-          <t>BTC-USD -14.87% · ETH-USD -15.74%</t>
+          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
         </is>
       </c>
       <c r="X248" t="inlineStr">
@@ -28837,7 +28837,7 @@
       </c>
       <c r="AC248" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.87% · ETH-USD -15.74%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
+          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD248" t="n">
@@ -28923,7 +28923,7 @@
       </c>
       <c r="W249" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X249" t="inlineStr">
@@ -28949,7 +28949,7 @@
       </c>
       <c r="AC249" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD249" t="n">
@@ -29035,7 +29035,7 @@
       </c>
       <c r="W250" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X250" t="inlineStr">
@@ -29061,7 +29061,7 @@
       </c>
       <c r="AC250" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD250" t="n">
@@ -29147,7 +29147,7 @@
       </c>
       <c r="W251" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X251" t="inlineStr">
@@ -29173,7 +29173,7 @@
       </c>
       <c r="AC251" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD251" t="n">
@@ -29259,7 +29259,7 @@
       </c>
       <c r="W252" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X252" t="inlineStr">
@@ -29285,7 +29285,7 @@
       </c>
       <c r="AC252" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD252" t="n">
@@ -29371,7 +29371,7 @@
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X253" t="inlineStr">
@@ -29397,7 +29397,7 @@
       </c>
       <c r="AC253" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD253" t="n">
@@ -29483,7 +29483,7 @@
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X254" t="inlineStr">
@@ -29509,7 +29509,7 @@
       </c>
       <c r="AC254" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD254" t="n">
@@ -29595,7 +29595,7 @@
       </c>
       <c r="W255" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X255" t="inlineStr">
@@ -29621,7 +29621,7 @@
       </c>
       <c r="AC255" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD255" t="n">
@@ -29707,7 +29707,7 @@
       </c>
       <c r="W256" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X256" t="inlineStr">
@@ -29733,7 +29733,7 @@
       </c>
       <c r="AC256" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD256" t="n">
@@ -29819,7 +29819,7 @@
       </c>
       <c r="W257" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X257" t="inlineStr">
@@ -29845,7 +29845,7 @@
       </c>
       <c r="AC257" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD257" t="n">
@@ -29931,7 +29931,7 @@
       </c>
       <c r="W258" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X258" t="inlineStr">
@@ -29957,7 +29957,7 @@
       </c>
       <c r="AC258" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD258" t="n">
@@ -30043,7 +30043,7 @@
       </c>
       <c r="W259" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X259" t="inlineStr">
@@ -30069,7 +30069,7 @@
       </c>
       <c r="AC259" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD259" t="n">
@@ -30155,7 +30155,7 @@
       </c>
       <c r="W260" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X260" t="inlineStr">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="AC260" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD260" t="n">
@@ -30267,7 +30267,7 @@
       </c>
       <c r="W261" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X261" t="inlineStr">
@@ -30293,7 +30293,7 @@
       </c>
       <c r="AC261" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD261" t="n">
@@ -30379,7 +30379,7 @@
       </c>
       <c r="W262" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X262" t="inlineStr">
@@ -30405,7 +30405,7 @@
       </c>
       <c r="AC262" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD262" t="n">
@@ -31731,7 +31731,7 @@
       </c>
       <c r="W274" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X274" t="inlineStr">
@@ -31757,7 +31757,7 @@
       </c>
       <c r="AC274" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Lejos del máximo 20D</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Lejos del máximo 20D</t>
         </is>
       </c>
       <c r="AD274" t="n">
@@ -31843,7 +31843,7 @@
       </c>
       <c r="W275" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.46%</t>
+          <t>XLE -10.08% · CL=F -21.42%</t>
         </is>
       </c>
       <c r="X275" t="inlineStr">
@@ -31869,7 +31869,7 @@
       </c>
       <c r="AC275" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.46%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD275" t="n">
@@ -31955,7 +31955,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>BTC-USD -14.87% · ETH-USD -15.74%</t>
+          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
         </is>
       </c>
       <c r="X276" t="inlineStr">
@@ -31981,7 +31981,7 @@
       </c>
       <c r="AC276" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.87% · ETH-USD -15.74%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD276" t="n">

</xml_diff>

<commit_message>
Actualizar analisis automatico BOT-ARQ v4.1
</commit_message>
<xml_diff>
--- a/analisis_acciones.xlsx
+++ b/analisis_acciones.xlsx
@@ -14683,7 +14683,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
+          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
         </is>
       </c>
       <c r="X124" t="inlineStr">
@@ -14713,7 +14713,7 @@
       </c>
       <c r="AC124" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD124" t="n">
@@ -14799,7 +14799,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
+          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
         </is>
       </c>
       <c r="X125" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="AC125" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; MACD sin confirmar; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; MACD sin confirmar; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD125" t="n">
@@ -14915,7 +14915,7 @@
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X126" t="inlineStr">
@@ -14945,7 +14945,7 @@
       </c>
       <c r="AC126" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD126" t="n">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X127" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="AC127" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD127" t="n">
@@ -18255,7 +18255,7 @@
       </c>
       <c r="W155" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X155" t="inlineStr">
@@ -18285,7 +18285,7 @@
       </c>
       <c r="AC155" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD155" t="n">
@@ -28023,7 +28023,7 @@
       </c>
       <c r="W241" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X241" t="inlineStr">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="AC241" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD241" t="n">
@@ -28139,7 +28139,7 @@
       </c>
       <c r="W242" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X242" t="inlineStr">
@@ -28165,7 +28165,7 @@
       </c>
       <c r="AC242" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Débil vs QQQ; Lejos del máximo 20D</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Débil vs QQQ; Lejos del máximo 20D</t>
         </is>
       </c>
       <c r="AD242" t="n">
@@ -28251,7 +28251,7 @@
       </c>
       <c r="W243" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X243" t="inlineStr">
@@ -28277,7 +28277,7 @@
       </c>
       <c r="AC243" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD243" t="n">
@@ -28363,7 +28363,7 @@
       </c>
       <c r="W244" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X244" t="inlineStr">
@@ -28389,7 +28389,7 @@
       </c>
       <c r="AC244" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD244" t="n">
@@ -28475,7 +28475,7 @@
       </c>
       <c r="W245" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X245" t="inlineStr">
@@ -28501,7 +28501,7 @@
       </c>
       <c r="AC245" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD245" t="n">
@@ -28587,7 +28587,7 @@
       </c>
       <c r="W246" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X246" t="inlineStr">
@@ -28613,7 +28613,7 @@
       </c>
       <c r="AC246" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD246" t="n">
@@ -28699,7 +28699,7 @@
       </c>
       <c r="W247" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X247" t="inlineStr">
@@ -28725,7 +28725,7 @@
       </c>
       <c r="AC247" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD247" t="n">
@@ -28811,7 +28811,7 @@
       </c>
       <c r="W248" t="inlineStr">
         <is>
-          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
+          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
         </is>
       </c>
       <c r="X248" t="inlineStr">
@@ -28837,7 +28837,7 @@
       </c>
       <c r="AC248" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
+          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD248" t="n">
@@ -28923,7 +28923,7 @@
       </c>
       <c r="W249" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X249" t="inlineStr">
@@ -28949,7 +28949,7 @@
       </c>
       <c r="AC249" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD249" t="n">
@@ -29035,7 +29035,7 @@
       </c>
       <c r="W250" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X250" t="inlineStr">
@@ -29061,7 +29061,7 @@
       </c>
       <c r="AC250" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD250" t="n">
@@ -29147,7 +29147,7 @@
       </c>
       <c r="W251" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X251" t="inlineStr">
@@ -29173,7 +29173,7 @@
       </c>
       <c r="AC251" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD251" t="n">
@@ -29259,7 +29259,7 @@
       </c>
       <c r="W252" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X252" t="inlineStr">
@@ -29285,7 +29285,7 @@
       </c>
       <c r="AC252" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD252" t="n">
@@ -29371,7 +29371,7 @@
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X253" t="inlineStr">
@@ -29397,7 +29397,7 @@
       </c>
       <c r="AC253" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD253" t="n">
@@ -29483,7 +29483,7 @@
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X254" t="inlineStr">
@@ -29509,7 +29509,7 @@
       </c>
       <c r="AC254" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD254" t="n">
@@ -29595,7 +29595,7 @@
       </c>
       <c r="W255" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X255" t="inlineStr">
@@ -29621,7 +29621,7 @@
       </c>
       <c r="AC255" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD255" t="n">
@@ -29707,7 +29707,7 @@
       </c>
       <c r="W256" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X256" t="inlineStr">
@@ -29733,7 +29733,7 @@
       </c>
       <c r="AC256" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD256" t="n">
@@ -29819,7 +29819,7 @@
       </c>
       <c r="W257" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X257" t="inlineStr">
@@ -29845,7 +29845,7 @@
       </c>
       <c r="AC257" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD257" t="n">
@@ -29931,7 +29931,7 @@
       </c>
       <c r="W258" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X258" t="inlineStr">
@@ -29957,7 +29957,7 @@
       </c>
       <c r="AC258" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD258" t="n">
@@ -30043,7 +30043,7 @@
       </c>
       <c r="W259" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X259" t="inlineStr">
@@ -30069,7 +30069,7 @@
       </c>
       <c r="AC259" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD259" t="n">
@@ -30155,7 +30155,7 @@
       </c>
       <c r="W260" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X260" t="inlineStr">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="AC260" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD260" t="n">
@@ -30267,7 +30267,7 @@
       </c>
       <c r="W261" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X261" t="inlineStr">
@@ -30293,7 +30293,7 @@
       </c>
       <c r="AC261" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD261" t="n">
@@ -30379,7 +30379,7 @@
       </c>
       <c r="W262" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X262" t="inlineStr">
@@ -30405,7 +30405,7 @@
       </c>
       <c r="AC262" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD262" t="n">
@@ -31731,7 +31731,7 @@
       </c>
       <c r="W274" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X274" t="inlineStr">
@@ -31757,7 +31757,7 @@
       </c>
       <c r="AC274" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Lejos del máximo 20D</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Lejos del máximo 20D</t>
         </is>
       </c>
       <c r="AD274" t="n">
@@ -31843,7 +31843,7 @@
       </c>
       <c r="W275" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X275" t="inlineStr">
@@ -31869,7 +31869,7 @@
       </c>
       <c r="AC275" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD275" t="n">
@@ -31955,7 +31955,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
+          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
         </is>
       </c>
       <c r="X276" t="inlineStr">
@@ -31981,7 +31981,7 @@
       </c>
       <c r="AC276" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD276" t="n">

</xml_diff>

<commit_message>
V4.2 CONFIGURACION REAL DEL MOTO
</commit_message>
<xml_diff>
--- a/analisis_acciones.xlsx
+++ b/analisis_acciones.xlsx
@@ -14683,7 +14683,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
+          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
         </is>
       </c>
       <c r="X124" t="inlineStr">
@@ -14713,7 +14713,7 @@
       </c>
       <c r="AC124" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD124" t="n">
@@ -14799,7 +14799,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
+          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
         </is>
       </c>
       <c r="X125" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="AC125" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; MACD sin confirmar; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; MACD sin confirmar; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD125" t="n">
@@ -14915,7 +14915,7 @@
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X126" t="inlineStr">
@@ -14945,7 +14945,7 @@
       </c>
       <c r="AC126" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD126" t="n">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X127" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="AC127" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD127" t="n">
@@ -18255,7 +18255,7 @@
       </c>
       <c r="W155" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X155" t="inlineStr">
@@ -18285,7 +18285,7 @@
       </c>
       <c r="AC155" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD155" t="n">
@@ -28023,7 +28023,7 @@
       </c>
       <c r="W241" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X241" t="inlineStr">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="AC241" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD241" t="n">
@@ -28139,7 +28139,7 @@
       </c>
       <c r="W242" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X242" t="inlineStr">
@@ -28165,7 +28165,7 @@
       </c>
       <c r="AC242" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Débil vs QQQ; Lejos del máximo 20D</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Débil vs QQQ; Lejos del máximo 20D</t>
         </is>
       </c>
       <c r="AD242" t="n">
@@ -28251,7 +28251,7 @@
       </c>
       <c r="W243" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X243" t="inlineStr">
@@ -28277,7 +28277,7 @@
       </c>
       <c r="AC243" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD243" t="n">
@@ -28363,7 +28363,7 @@
       </c>
       <c r="W244" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X244" t="inlineStr">
@@ -28389,7 +28389,7 @@
       </c>
       <c r="AC244" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD244" t="n">
@@ -28475,7 +28475,7 @@
       </c>
       <c r="W245" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X245" t="inlineStr">
@@ -28501,7 +28501,7 @@
       </c>
       <c r="AC245" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD245" t="n">
@@ -28587,7 +28587,7 @@
       </c>
       <c r="W246" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X246" t="inlineStr">
@@ -28613,7 +28613,7 @@
       </c>
       <c r="AC246" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD246" t="n">
@@ -28699,7 +28699,7 @@
       </c>
       <c r="W247" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X247" t="inlineStr">
@@ -28725,7 +28725,7 @@
       </c>
       <c r="AC247" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD247" t="n">
@@ -28811,7 +28811,7 @@
       </c>
       <c r="W248" t="inlineStr">
         <is>
-          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
+          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
         </is>
       </c>
       <c r="X248" t="inlineStr">
@@ -28837,7 +28837,7 @@
       </c>
       <c r="AC248" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
+          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD248" t="n">
@@ -28923,7 +28923,7 @@
       </c>
       <c r="W249" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X249" t="inlineStr">
@@ -28949,7 +28949,7 @@
       </c>
       <c r="AC249" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD249" t="n">
@@ -29035,7 +29035,7 @@
       </c>
       <c r="W250" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X250" t="inlineStr">
@@ -29061,7 +29061,7 @@
       </c>
       <c r="AC250" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD250" t="n">
@@ -29147,7 +29147,7 @@
       </c>
       <c r="W251" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X251" t="inlineStr">
@@ -29173,7 +29173,7 @@
       </c>
       <c r="AC251" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD251" t="n">
@@ -29259,7 +29259,7 @@
       </c>
       <c r="W252" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X252" t="inlineStr">
@@ -29285,7 +29285,7 @@
       </c>
       <c r="AC252" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD252" t="n">
@@ -29371,7 +29371,7 @@
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X253" t="inlineStr">
@@ -29397,7 +29397,7 @@
       </c>
       <c r="AC253" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD253" t="n">
@@ -29483,7 +29483,7 @@
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X254" t="inlineStr">
@@ -29509,7 +29509,7 @@
       </c>
       <c r="AC254" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD254" t="n">
@@ -29595,7 +29595,7 @@
       </c>
       <c r="W255" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X255" t="inlineStr">
@@ -29621,7 +29621,7 @@
       </c>
       <c r="AC255" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD255" t="n">
@@ -29707,7 +29707,7 @@
       </c>
       <c r="W256" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X256" t="inlineStr">
@@ -29733,7 +29733,7 @@
       </c>
       <c r="AC256" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD256" t="n">
@@ -29819,7 +29819,7 @@
       </c>
       <c r="W257" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X257" t="inlineStr">
@@ -29845,7 +29845,7 @@
       </c>
       <c r="AC257" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD257" t="n">
@@ -29931,7 +29931,7 @@
       </c>
       <c r="W258" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X258" t="inlineStr">
@@ -29957,7 +29957,7 @@
       </c>
       <c r="AC258" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD258" t="n">
@@ -30043,7 +30043,7 @@
       </c>
       <c r="W259" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X259" t="inlineStr">
@@ -30069,7 +30069,7 @@
       </c>
       <c r="AC259" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD259" t="n">
@@ -30155,7 +30155,7 @@
       </c>
       <c r="W260" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X260" t="inlineStr">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="AC260" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD260" t="n">
@@ -30267,7 +30267,7 @@
       </c>
       <c r="W261" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X261" t="inlineStr">
@@ -30293,7 +30293,7 @@
       </c>
       <c r="AC261" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD261" t="n">
@@ -30379,7 +30379,7 @@
       </c>
       <c r="W262" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X262" t="inlineStr">
@@ -30405,7 +30405,7 @@
       </c>
       <c r="AC262" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD262" t="n">
@@ -31731,7 +31731,7 @@
       </c>
       <c r="W274" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X274" t="inlineStr">
@@ -31757,7 +31757,7 @@
       </c>
       <c r="AC274" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Lejos del máximo 20D</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Lejos del máximo 20D</t>
         </is>
       </c>
       <c r="AD274" t="n">
@@ -31843,7 +31843,7 @@
       </c>
       <c r="W275" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.42%</t>
+          <t>XLE -10.08% · CL=F -21.16%</t>
         </is>
       </c>
       <c r="X275" t="inlineStr">
@@ -31869,7 +31869,7 @@
       </c>
       <c r="AC275" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.42%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD275" t="n">
@@ -31955,7 +31955,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>BTC-USD -14.91% · ETH-USD -15.63%</t>
+          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
         </is>
       </c>
       <c r="X276" t="inlineStr">
@@ -31981,7 +31981,7 @@
       </c>
       <c r="AC276" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.91% · ETH-USD -15.63%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD276" t="n">

</xml_diff>

<commit_message>
Actualizar analisis automatico BOT-ARQ v4.2
</commit_message>
<xml_diff>
--- a/analisis_acciones.xlsx
+++ b/analisis_acciones.xlsx
@@ -14683,7 +14683,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
+          <t>BTC-USD -14.64% · ETH-USD -15.42%</t>
         </is>
       </c>
       <c r="X124" t="inlineStr">
@@ -14713,7 +14713,7 @@
       </c>
       <c r="AC124" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.64% · ETH-USD -15.42%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD124" t="n">
@@ -14799,7 +14799,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
+          <t>BTC-USD -14.64% · ETH-USD -15.42%</t>
         </is>
       </c>
       <c r="X125" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="AC125" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; MACD sin confirmar; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.64% · ETH-USD -15.42%; MACD sin confirmar; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD125" t="n">
@@ -14915,7 +14915,7 @@
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X126" t="inlineStr">
@@ -14945,7 +14945,7 @@
       </c>
       <c r="AC126" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD126" t="n">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X127" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="AC127" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD127" t="n">
@@ -18255,7 +18255,7 @@
       </c>
       <c r="W155" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X155" t="inlineStr">
@@ -18285,7 +18285,7 @@
       </c>
       <c r="AC155" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Subida muy extendida 5D; Muy alejada de MA20; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD155" t="n">
@@ -28023,7 +28023,7 @@
       </c>
       <c r="W241" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X241" t="inlineStr">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="AC241" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD241" t="n">
@@ -28139,7 +28139,7 @@
       </c>
       <c r="W242" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X242" t="inlineStr">
@@ -28165,7 +28165,7 @@
       </c>
       <c r="AC242" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Débil vs QQQ; Lejos del máximo 20D</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Débil vs QQQ; Lejos del máximo 20D</t>
         </is>
       </c>
       <c r="AD242" t="n">
@@ -28251,7 +28251,7 @@
       </c>
       <c r="W243" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X243" t="inlineStr">
@@ -28277,7 +28277,7 @@
       </c>
       <c r="AC243" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD243" t="n">
@@ -28363,7 +28363,7 @@
       </c>
       <c r="W244" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X244" t="inlineStr">
@@ -28389,7 +28389,7 @@
       </c>
       <c r="AC244" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD244" t="n">
@@ -28475,7 +28475,7 @@
       </c>
       <c r="W245" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X245" t="inlineStr">
@@ -28501,7 +28501,7 @@
       </c>
       <c r="AC245" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD245" t="n">
@@ -28587,7 +28587,7 @@
       </c>
       <c r="W246" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X246" t="inlineStr">
@@ -28613,7 +28613,7 @@
       </c>
       <c r="AC246" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD246" t="n">
@@ -28699,7 +28699,7 @@
       </c>
       <c r="W247" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X247" t="inlineStr">
@@ -28725,7 +28725,7 @@
       </c>
       <c r="AC247" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD247" t="n">
@@ -28811,7 +28811,7 @@
       </c>
       <c r="W248" t="inlineStr">
         <is>
-          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
+          <t>BTC-USD -14.64% · ETH-USD -15.42%</t>
         </is>
       </c>
       <c r="X248" t="inlineStr">
@@ -28837,7 +28837,7 @@
       </c>
       <c r="AC248" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
+          <t>Sector no acompaña: BTC-USD -14.64% · ETH-USD -15.42%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD248" t="n">
@@ -28923,7 +28923,7 @@
       </c>
       <c r="W249" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X249" t="inlineStr">
@@ -28949,7 +28949,7 @@
       </c>
       <c r="AC249" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD249" t="n">
@@ -29035,7 +29035,7 @@
       </c>
       <c r="W250" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X250" t="inlineStr">
@@ -29061,7 +29061,7 @@
       </c>
       <c r="AC250" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD250" t="n">
@@ -29147,7 +29147,7 @@
       </c>
       <c r="W251" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X251" t="inlineStr">
@@ -29173,7 +29173,7 @@
       </c>
       <c r="AC251" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD251" t="n">
@@ -29259,7 +29259,7 @@
       </c>
       <c r="W252" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X252" t="inlineStr">
@@ -29285,7 +29285,7 @@
       </c>
       <c r="AC252" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD252" t="n">
@@ -29371,7 +29371,7 @@
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X253" t="inlineStr">
@@ -29397,7 +29397,7 @@
       </c>
       <c r="AC253" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD253" t="n">
@@ -29483,7 +29483,7 @@
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X254" t="inlineStr">
@@ -29509,7 +29509,7 @@
       </c>
       <c r="AC254" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD254" t="n">
@@ -29595,7 +29595,7 @@
       </c>
       <c r="W255" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X255" t="inlineStr">
@@ -29621,7 +29621,7 @@
       </c>
       <c r="AC255" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD255" t="n">
@@ -29707,7 +29707,7 @@
       </c>
       <c r="W256" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X256" t="inlineStr">
@@ -29733,7 +29733,7 @@
       </c>
       <c r="AC256" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD256" t="n">
@@ -29819,7 +29819,7 @@
       </c>
       <c r="W257" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X257" t="inlineStr">
@@ -29845,7 +29845,7 @@
       </c>
       <c r="AC257" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; MACD sin confirmar; Momentum negativo; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD257" t="n">
@@ -29931,7 +29931,7 @@
       </c>
       <c r="W258" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X258" t="inlineStr">
@@ -29957,7 +29957,7 @@
       </c>
       <c r="AC258" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD258" t="n">
@@ -30043,7 +30043,7 @@
       </c>
       <c r="W259" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X259" t="inlineStr">
@@ -30069,7 +30069,7 @@
       </c>
       <c r="AC259" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD259" t="n">
@@ -30155,7 +30155,7 @@
       </c>
       <c r="W260" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X260" t="inlineStr">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="AC260" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD260" t="n">
@@ -30267,7 +30267,7 @@
       </c>
       <c r="W261" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X261" t="inlineStr">
@@ -30293,7 +30293,7 @@
       </c>
       <c r="AC261" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD261" t="n">
@@ -30379,7 +30379,7 @@
       </c>
       <c r="W262" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X262" t="inlineStr">
@@ -30405,7 +30405,7 @@
       </c>
       <c r="AC262" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD262" t="n">
@@ -31731,7 +31731,7 @@
       </c>
       <c r="W274" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X274" t="inlineStr">
@@ -31757,7 +31757,7 @@
       </c>
       <c r="AC274" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Lejos del máximo 20D</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Lejos del máximo 20D</t>
         </is>
       </c>
       <c r="AD274" t="n">
@@ -31843,7 +31843,7 @@
       </c>
       <c r="W275" t="inlineStr">
         <is>
-          <t>XLE -10.08% · CL=F -21.16%</t>
+          <t>XLE -10.08% · CL=F -20.64%</t>
         </is>
       </c>
       <c r="X275" t="inlineStr">
@@ -31869,7 +31869,7 @@
       </c>
       <c r="AC275" t="inlineStr">
         <is>
-          <t>Sector no acompaña: XLE -10.08% · CL=F -21.16%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
+          <t>Sector no acompaña: XLE -10.08% · CL=F -20.64%; Precio bajo MA20; RSI débil; MACD sin confirmar; Momentum negativo</t>
         </is>
       </c>
       <c r="AD275" t="n">
@@ -31955,7 +31955,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>BTC-USD -14.97% · ETH-USD -15.68%</t>
+          <t>BTC-USD -14.64% · ETH-USD -15.42%</t>
         </is>
       </c>
       <c r="X276" t="inlineStr">
@@ -31981,7 +31981,7 @@
       </c>
       <c r="AC276" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.97% · ETH-USD -15.68%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: BTC-USD -14.64% · ETH-USD -15.42%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD276" t="n">

</xml_diff>

<commit_message>
Actualizar analisis automatico BOT-ARQ v4.4.1
</commit_message>
<xml_diff>
--- a/analisis_acciones.xlsx
+++ b/analisis_acciones.xlsx
@@ -14791,7 +14791,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>BTC-USD -14.22% · ETH-USD -15.6%</t>
+          <t>BTC-USD -14.15% · ETH-USD -15.51%</t>
         </is>
       </c>
       <c r="X125" t="inlineStr">
@@ -14821,7 +14821,7 @@
       </c>
       <c r="AC125" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.22% · ETH-USD -15.6%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.15% · ETH-USD -15.51%; MACD sin confirmar; Momentum 5D extendido; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD125" t="n">
@@ -14907,7 +14907,7 @@
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>BTC-USD -14.22% · ETH-USD -15.6%</t>
+          <t>BTC-USD -14.15% · ETH-USD -15.51%</t>
         </is>
       </c>
       <c r="X126" t="inlineStr">
@@ -14937,7 +14937,7 @@
       </c>
       <c r="AC126" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.22% · ETH-USD -15.6%; MACD sin confirmar; Volatilidad alta</t>
+          <t>Sector no acompaña: BTC-USD -14.15% · ETH-USD -15.51%; MACD sin confirmar; Volatilidad alta</t>
         </is>
       </c>
       <c r="AD126" t="n">
@@ -28567,7 +28567,7 @@
       </c>
       <c r="W246" t="inlineStr">
         <is>
-          <t>BTC-USD -14.22% · ETH-USD -15.6%</t>
+          <t>BTC-USD -14.15% · ETH-USD -15.51%</t>
         </is>
       </c>
       <c r="X246" t="inlineStr">
@@ -28593,7 +28593,7 @@
       </c>
       <c r="AC246" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.22% · ETH-USD -15.6%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
+          <t>Sector no acompaña: BTC-USD -14.15% · ETH-USD -15.51%; Precio bajo MA20; Tendencia larga débil; RSI débil; Débil vs QQQ</t>
         </is>
       </c>
       <c r="AD246" t="n">
@@ -31935,7 +31935,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>BTC-USD -14.22% · ETH-USD -15.6%</t>
+          <t>BTC-USD -14.15% · ETH-USD -15.51%</t>
         </is>
       </c>
       <c r="X276" t="inlineStr">
@@ -31961,7 +31961,7 @@
       </c>
       <c r="AC276" t="inlineStr">
         <is>
-          <t>Sector no acompaña: BTC-USD -14.22% · ETH-USD -15.6%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
+          <t>Sector no acompaña: BTC-USD -14.15% · ETH-USD -15.51%; Precio bajo MA20; Tendencia larga débil; RSI débil; MACD sin confirmar</t>
         </is>
       </c>
       <c r="AD276" t="n">

</xml_diff>